<commit_message>
Update live college page audit Excel dashboard
</commit_message>
<xml_diff>
--- a/college-page-audit-dashboard.xlsx
+++ b/college-page-audit-dashboard.xlsx
@@ -614,7 +614,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18 UTC</t>
+          <t>2026-09-01 13:08:38 UTC</t>
         </is>
       </c>
       <c r="C7" s="3" t="n"/>
@@ -6140,7 +6140,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -6172,7 +6172,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -6204,7 +6204,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -6236,7 +6236,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -6268,7 +6268,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -6300,7 +6300,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -6332,7 +6332,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -6364,7 +6364,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -6396,7 +6396,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -6428,7 +6428,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -6460,7 +6460,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -6492,7 +6492,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -6524,7 +6524,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -6556,7 +6556,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -6588,7 +6588,7 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -6620,7 +6620,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -6652,7 +6652,7 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -6684,7 +6684,7 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -6716,7 +6716,7 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -6748,7 +6748,7 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -6780,7 +6780,7 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -6812,7 +6812,7 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -6844,7 +6844,7 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -6876,7 +6876,7 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -6908,7 +6908,7 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -6940,7 +6940,7 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -6972,7 +6972,7 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -7004,7 +7004,7 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -7036,7 +7036,7 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -7068,7 +7068,7 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -7100,7 +7100,7 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -7132,7 +7132,7 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -7164,7 +7164,7 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -7196,7 +7196,7 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -7228,7 +7228,7 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -7260,7 +7260,7 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -7292,7 +7292,7 @@
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -7324,7 +7324,7 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -7356,7 +7356,7 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -7388,7 +7388,7 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -7420,7 +7420,7 @@
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -7452,7 +7452,7 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -7484,7 +7484,7 @@
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -7516,7 +7516,7 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -7548,7 +7548,7 @@
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -7580,7 +7580,7 @@
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -7612,7 +7612,7 @@
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -7644,7 +7644,7 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -7676,7 +7676,7 @@
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -7708,7 +7708,7 @@
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -7740,7 +7740,7 @@
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
@@ -7772,7 +7772,7 @@
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
@@ -7804,7 +7804,7 @@
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
@@ -7836,7 +7836,7 @@
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
@@ -7868,7 +7868,7 @@
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
@@ -7900,7 +7900,7 @@
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
@@ -7932,7 +7932,7 @@
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
@@ -7964,7 +7964,7 @@
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
@@ -7996,7 +7996,7 @@
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
@@ -8028,7 +8028,7 @@
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
@@ -8060,7 +8060,7 @@
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
@@ -8092,7 +8092,7 @@
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01:18</t>
+          <t>2026-09-01 13:08:38</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update live college page audit dashboards
</commit_message>
<xml_diff>
--- a/college-page-audit-dashboard.xlsx
+++ b/college-page-audit-dashboard.xlsx
@@ -614,7 +614,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11 UTC</t>
+          <t>2026-09-01 14:54:46 UTC</t>
         </is>
       </c>
       <c r="C7" s="3" t="n"/>
@@ -842,7 +842,7 @@
       </c>
       <c r="O2" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P2" s="3" t="n">
@@ -1000,7 +1000,7 @@
       </c>
       <c r="O4" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P4" s="3" t="n">
@@ -1080,7 +1080,7 @@
       </c>
       <c r="O5" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P5" s="3" t="n">
@@ -1160,7 +1160,7 @@
       </c>
       <c r="O6" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P6" s="3" t="n">
@@ -1240,7 +1240,7 @@
       </c>
       <c r="O7" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P7" s="3" t="n">
@@ -1632,7 +1632,7 @@
       </c>
       <c r="O12" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P12" s="3" t="n">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="O13" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P13" s="3" t="n">
@@ -1792,7 +1792,7 @@
       </c>
       <c r="O14" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P14" s="3" t="n">
@@ -1872,7 +1872,7 @@
       </c>
       <c r="O15" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P15" s="3" t="n">
@@ -1952,7 +1952,7 @@
       </c>
       <c r="O16" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P16" s="3" t="n">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="O17" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P17" s="3" t="n">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="O18" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P18" s="3" t="n">
@@ -2192,7 +2192,7 @@
       </c>
       <c r="O19" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P19" s="3" t="n">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="O20" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P20" s="3" t="n">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="O21" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P21" s="3" t="n">
@@ -2432,7 +2432,7 @@
       </c>
       <c r="O22" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P22" s="3" t="n">
@@ -2512,7 +2512,7 @@
       </c>
       <c r="O23" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P23" s="3" t="n">
@@ -2592,7 +2592,7 @@
       </c>
       <c r="O24" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P24" s="3" t="n">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="O25" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P25" s="3" t="n">
@@ -2752,7 +2752,7 @@
       </c>
       <c r="O26" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P26" s="3" t="n">
@@ -2832,7 +2832,7 @@
       </c>
       <c r="O27" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P27" s="3" t="n">
@@ -2912,7 +2912,7 @@
       </c>
       <c r="O28" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P28" s="3" t="n">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="O29" s="3" t="inlineStr">
         <is>
-          <t>177b0783bd532325a4bdb74ec3bea6882107d82c</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P29" s="3" t="n">
@@ -3072,7 +3072,7 @@
       </c>
       <c r="O30" s="3" t="inlineStr">
         <is>
-          <t>177b0783bd532325a4bdb74ec3bea6882107d82c</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P30" s="3" t="n">
@@ -3152,7 +3152,7 @@
       </c>
       <c r="O31" s="3" t="inlineStr">
         <is>
-          <t>f08f120663283a98f388c101b35fe67b6b41a1e8</t>
+          <t>07e4e3a8409edbf9ba4ea107629d1281c6ce56b3</t>
         </is>
       </c>
       <c r="P31" s="3" t="n">
@@ -3232,7 +3232,7 @@
       </c>
       <c r="O32" s="3" t="inlineStr">
         <is>
-          <t>177b0783bd532325a4bdb74ec3bea6882107d82c</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P32" s="3" t="n">
@@ -3307,16 +3307,16 @@
       </c>
       <c r="N33" s="3" t="inlineStr">
         <is>
-          <t>Content audit: 4 issue group(s)</t>
+          <t>Content audit: 3 issue group(s)</t>
         </is>
       </c>
       <c r="O33" s="3" t="inlineStr">
         <is>
-          <t>06e3c0a719c42bbb7ae22e9fa2c7ff5297543fb0</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P33" s="3" t="n">
-        <v>67</v>
+        <v>82</v>
       </c>
     </row>
     <row r="34">
@@ -3392,7 +3392,7 @@
       </c>
       <c r="O34" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P34" s="3" t="n">
@@ -3472,7 +3472,7 @@
       </c>
       <c r="O35" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P35" s="3" t="n">
@@ -3552,7 +3552,7 @@
       </c>
       <c r="O36" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P36" s="3" t="n">
@@ -3632,7 +3632,7 @@
       </c>
       <c r="O37" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P37" s="3" t="n">
@@ -3712,7 +3712,7 @@
       </c>
       <c r="O38" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P38" s="3" t="n">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="O39" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P39" s="3" t="n">
@@ -3872,7 +3872,7 @@
       </c>
       <c r="O40" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P40" s="3" t="n">
@@ -3952,7 +3952,7 @@
       </c>
       <c r="O41" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P41" s="3" t="n">
@@ -4032,7 +4032,7 @@
       </c>
       <c r="O42" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P42" s="3" t="n">
@@ -4112,7 +4112,7 @@
       </c>
       <c r="O43" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P43" s="3" t="n">
@@ -4192,7 +4192,7 @@
       </c>
       <c r="O44" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P44" s="3" t="n">
@@ -4272,7 +4272,7 @@
       </c>
       <c r="O45" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P45" s="3" t="n">
@@ -4352,7 +4352,7 @@
       </c>
       <c r="O46" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P46" s="3" t="n">
@@ -4432,7 +4432,7 @@
       </c>
       <c r="O47" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P47" s="3" t="n">
@@ -4512,7 +4512,7 @@
       </c>
       <c r="O48" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P48" s="3" t="n">
@@ -4592,7 +4592,7 @@
       </c>
       <c r="O49" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P49" s="3" t="n">
@@ -4672,7 +4672,7 @@
       </c>
       <c r="O50" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P50" s="3" t="n">
@@ -4752,7 +4752,7 @@
       </c>
       <c r="O51" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P51" s="3" t="n">
@@ -4832,7 +4832,7 @@
       </c>
       <c r="O52" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P52" s="3" t="n">
@@ -4912,7 +4912,7 @@
       </c>
       <c r="O53" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P53" s="3" t="n">
@@ -4992,7 +4992,7 @@
       </c>
       <c r="O54" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P54" s="3" t="n">
@@ -5072,7 +5072,7 @@
       </c>
       <c r="O55" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P55" s="3" t="n">
@@ -5152,7 +5152,7 @@
       </c>
       <c r="O56" s="3" t="inlineStr">
         <is>
-          <t>5a6cb849ab8506d311a79168f1cc799bcfeff8d6</t>
+          <t>07e4e3a8409edbf9ba4ea107629d1281c6ce56b3</t>
         </is>
       </c>
       <c r="P56" s="3" t="n">
@@ -5232,7 +5232,7 @@
       </c>
       <c r="O57" s="3" t="inlineStr">
         <is>
-          <t>f2555c17065d8fd39462b393be368faa5e6c9865</t>
+          <t>07e4e3a8409edbf9ba4ea107629d1281c6ce56b3</t>
         </is>
       </c>
       <c r="P57" s="3" t="n">
@@ -5312,7 +5312,7 @@
       </c>
       <c r="O58" s="3" t="inlineStr">
         <is>
-          <t>c93a9249f83f53be8a0f5c4ec928241cfd399e40</t>
+          <t>07e4e3a8409edbf9ba4ea107629d1281c6ce56b3</t>
         </is>
       </c>
       <c r="P58" s="3" t="n">
@@ -5392,11 +5392,11 @@
       </c>
       <c r="O59" s="3" t="inlineStr">
         <is>
-          <t>610946ef955c6ef9cbf71d15167e817cee584084</t>
+          <t>07e4e3a8409edbf9ba4ea107629d1281c6ce56b3</t>
         </is>
       </c>
       <c r="P59" s="3" t="n">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="60">
@@ -5472,7 +5472,7 @@
       </c>
       <c r="O60" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P60" s="3" t="n">
@@ -5552,7 +5552,7 @@
       </c>
       <c r="O61" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P61" s="3" t="n">
@@ -5632,7 +5632,7 @@
       </c>
       <c r="O62" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P62" s="3" t="n">
@@ -5712,7 +5712,7 @@
       </c>
       <c r="O63" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P63" s="3" t="n">
@@ -5792,7 +5792,7 @@
       </c>
       <c r="O64" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P64" s="3" t="n">
@@ -5872,7 +5872,7 @@
       </c>
       <c r="O65" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P65" s="3" t="n">
@@ -5952,7 +5952,7 @@
       </c>
       <c r="O66" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P66" s="3" t="n">
@@ -6032,7 +6032,7 @@
       </c>
       <c r="O67" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
       <c r="P67" s="3" t="n">
@@ -6460,7 +6460,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -6485,14 +6485,14 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -6524,7 +6524,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -6549,14 +6549,14 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -6581,14 +6581,14 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -6613,14 +6613,14 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -6645,14 +6645,14 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -6684,7 +6684,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -6716,7 +6716,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -6748,7 +6748,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -6780,7 +6780,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -6805,14 +6805,14 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -6837,14 +6837,14 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -6869,14 +6869,14 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -6901,14 +6901,14 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -6933,14 +6933,14 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -6965,14 +6965,14 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -6997,14 +6997,14 @@
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -7029,14 +7029,14 @@
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -7061,14 +7061,14 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -7093,14 +7093,14 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -7125,14 +7125,14 @@
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -7157,14 +7157,14 @@
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -7189,14 +7189,14 @@
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -7221,14 +7221,14 @@
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -7253,14 +7253,14 @@
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -7285,14 +7285,14 @@
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -7317,14 +7317,14 @@
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -7349,14 +7349,14 @@
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>177b0783bd532325a4bdb74ec3bea6882107d82c</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -7381,14 +7381,14 @@
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>177b0783bd532325a4bdb74ec3bea6882107d82c</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -7413,14 +7413,14 @@
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>f08f120663283a98f388c101b35fe67b6b41a1e8</t>
+          <t>07e4e3a8409edbf9ba4ea107629d1281c6ce56b3</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -7445,14 +7445,14 @@
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>177b0783bd532325a4bdb74ec3bea6882107d82c</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -7477,14 +7477,14 @@
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>06e3c0a719c42bbb7ae22e9fa2c7ff5297543fb0</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -7509,14 +7509,14 @@
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -7541,14 +7541,14 @@
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -7573,14 +7573,14 @@
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -7605,14 +7605,14 @@
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -7637,14 +7637,14 @@
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -7669,14 +7669,14 @@
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -7701,14 +7701,14 @@
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -7733,14 +7733,14 @@
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -7765,14 +7765,14 @@
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -7797,14 +7797,14 @@
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -7829,14 +7829,14 @@
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -7861,14 +7861,14 @@
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -7893,14 +7893,14 @@
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -7925,14 +7925,14 @@
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -7957,14 +7957,14 @@
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -7989,14 +7989,14 @@
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -8021,14 +8021,14 @@
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -8053,14 +8053,14 @@
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
@@ -8085,14 +8085,14 @@
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
@@ -8117,14 +8117,14 @@
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
@@ -8149,14 +8149,14 @@
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
@@ -8181,14 +8181,14 @@
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
@@ -8213,14 +8213,14 @@
       </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>5a6cb849ab8506d311a79168f1cc799bcfeff8d6</t>
+          <t>07e4e3a8409edbf9ba4ea107629d1281c6ce56b3</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
@@ -8245,14 +8245,14 @@
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>f2555c17065d8fd39462b393be368faa5e6c9865</t>
+          <t>07e4e3a8409edbf9ba4ea107629d1281c6ce56b3</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
@@ -8277,14 +8277,14 @@
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>c93a9249f83f53be8a0f5c4ec928241cfd399e40</t>
+          <t>07e4e3a8409edbf9ba4ea107629d1281c6ce56b3</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
@@ -8309,14 +8309,14 @@
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>610946ef955c6ef9cbf71d15167e817cee584084</t>
+          <t>07e4e3a8409edbf9ba4ea107629d1281c6ce56b3</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
@@ -8341,14 +8341,14 @@
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
@@ -8373,14 +8373,14 @@
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
@@ -8405,14 +8405,14 @@
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
@@ -8437,14 +8437,14 @@
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
@@ -8469,14 +8469,14 @@
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
@@ -8501,14 +8501,14 @@
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
@@ -8533,14 +8533,14 @@
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>2026-09-01 14:40:11</t>
+          <t>2026-09-01 14:54:46</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
@@ -8565,7 +8565,7 @@
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>a9099bb08d703c457fafa8abbf8f3636c14c7362</t>
+          <t>85004d33d5504ba979316c9440c90ae5b109614f</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update live college audit and production trackers
</commit_message>
<xml_diff>
--- a/college-page-audit-dashboard.xlsx
+++ b/college-page-audit-dashboard.xlsx
@@ -614,7 +614,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11 UTC</t>
+          <t>2026-09-02 07:46:28 UTC</t>
         </is>
       </c>
       <c r="C7" s="3" t="n"/>
@@ -6470,7 +6470,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -6502,7 +6502,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -6534,7 +6534,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -6566,7 +6566,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -6598,7 +6598,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -6630,7 +6630,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -6662,7 +6662,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -6694,7 +6694,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -6726,7 +6726,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -6758,7 +6758,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -6790,7 +6790,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -6822,7 +6822,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -6854,7 +6854,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -6886,7 +6886,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -6918,7 +6918,7 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -6950,7 +6950,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -6982,7 +6982,7 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -7014,7 +7014,7 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -7046,7 +7046,7 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -7078,7 +7078,7 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -7110,7 +7110,7 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -7142,7 +7142,7 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -7174,7 +7174,7 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -7206,7 +7206,7 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -7238,7 +7238,7 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -7270,7 +7270,7 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -7302,7 +7302,7 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -7334,7 +7334,7 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -7366,7 +7366,7 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -7398,7 +7398,7 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -7430,7 +7430,7 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -7462,7 +7462,7 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -7494,7 +7494,7 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -7526,7 +7526,7 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -7558,7 +7558,7 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -7590,7 +7590,7 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -7622,7 +7622,7 @@
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -7654,7 +7654,7 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -7686,7 +7686,7 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -7718,7 +7718,7 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -7750,7 +7750,7 @@
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -7782,7 +7782,7 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -7814,7 +7814,7 @@
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -7846,7 +7846,7 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -7878,7 +7878,7 @@
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -7910,7 +7910,7 @@
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -7942,7 +7942,7 @@
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -7974,7 +7974,7 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -8006,7 +8006,7 @@
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -8038,7 +8038,7 @@
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -8070,7 +8070,7 @@
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
@@ -8102,7 +8102,7 @@
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
@@ -8134,7 +8134,7 @@
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
@@ -8166,7 +8166,7 @@
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
@@ -8198,7 +8198,7 @@
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
@@ -8230,7 +8230,7 @@
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
@@ -8262,7 +8262,7 @@
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
@@ -8294,7 +8294,7 @@
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
@@ -8326,7 +8326,7 @@
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
@@ -8358,7 +8358,7 @@
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
@@ -8390,7 +8390,7 @@
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
@@ -8422,7 +8422,7 @@
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
@@ -8454,7 +8454,7 @@
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
@@ -8486,7 +8486,7 @@
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
@@ -8518,7 +8518,7 @@
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
@@ -8550,7 +8550,7 @@
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>2026-09-02 07:14:11</t>
+          <t>2026-09-02 07:46:28</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">

</xml_diff>